<commit_message>
Update BOM. example code
</commit_message>
<xml_diff>
--- a/Electrical/miniBCS-4_J005904.xlsx
+++ b/Electrical/miniBCS-4_J005904.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sawtelles\Documents\GitHub\miniBSC-4\Electrical\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C57F6CF-8BA7-4C58-9A36-0193E1BE2BFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5E0C213-35BC-4921-A31A-F7A5831E428F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6780" yWindow="615" windowWidth="30225" windowHeight="14250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1140" yWindow="600" windowWidth="29490" windowHeight="14445" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="J005904_miniBCSrevG" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="228">
   <si>
     <t>Qty</t>
   </si>
@@ -709,6 +709,15 @@
   </si>
   <si>
     <t>296-SN74LVC2G17DBVRCT-ND</t>
+  </si>
+  <si>
+    <t>J11</t>
+  </si>
+  <si>
+    <t>U2 U8</t>
+  </si>
+  <si>
+    <t>J26</t>
   </si>
 </sst>
 </file>
@@ -2808,6 +2817,9 @@
       <c r="C45" t="s">
         <v>175</v>
       </c>
+      <c r="D45" s="1" t="s">
+        <v>46</v>
+      </c>
       <c r="E45" s="1" t="s">
         <v>167</v>
       </c>
@@ -2835,6 +2847,9 @@
       <c r="C46" t="s">
         <v>209</v>
       </c>
+      <c r="D46" s="1" t="s">
+        <v>227</v>
+      </c>
       <c r="E46" s="1" t="s">
         <v>211</v>
       </c>
@@ -2862,6 +2877,9 @@
       <c r="C47" t="s">
         <v>216</v>
       </c>
+      <c r="D47" s="1" t="s">
+        <v>225</v>
+      </c>
       <c r="E47" s="1" t="s">
         <v>218</v>
       </c>
@@ -2888,6 +2906,9 @@
       </c>
       <c r="C48" t="s">
         <v>220</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>226</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>223</v>

</xml_diff>